<commit_message>
chore: remove image/reel pattern, update cron, and isolate cloudinary folder
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Repost Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="State" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repost Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1176,6 +1176,141 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>dua</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DYEBevkEgW-</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-05-11 19:28:59 UTC</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DYEBevkEgW-/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>lifestyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DX1E7SAK46i</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>reel</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-05-11 19:31:54 UTC</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DX1E7SAK46i/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DYGuEWpE4oj</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-05-11 19:33:17 UTC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DYGuEWpE4oj/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>motivation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DJ4DQK_TH23</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-05-11 19:41:08 UTC</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DJ4DQK_TH23/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DXwVc-pq6td</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>reel</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-05-11 19:45:51 UTC</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DXwVc-pq6td/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>general</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1348,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>reel</t>
+          <t>image</t>
         </is>
       </c>
     </row>

</xml_diff>